<commit_message>
Updated group list for GDV4000
</commit_message>
<xml_diff>
--- a/T2/GDV4000/GDV4000_25_26_Groups.xlsx
+++ b/T2/GDV4000/GDV4000_25_26_Groups.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ian\TEACHING_25_26\2025_26\T2\GDV4000\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A77759F2-95B2-48D2-9683-2DF27C0908FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2476AA7C-ABEE-465A-97E3-97588E3E4E90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="82440" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{587E5374-C9D8-4859-B380-F0EE43715D22}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="63">
   <si>
     <t>Team Member Name</t>
   </si>
@@ -213,13 +213,25 @@
   </si>
   <si>
     <t>Benji Fowler</t>
+  </si>
+  <si>
+    <t>Poss Transferring from Course</t>
+  </si>
+  <si>
+    <t>Emailed 24/02/26 Due to lack of attendance</t>
+  </si>
+  <si>
+    <t>Responded - Has been ill but will be in.</t>
+  </si>
+  <si>
+    <t>Still awaiting to hear</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -235,8 +247,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -306,6 +325,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -331,7 +356,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -365,6 +390,11 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -699,16 +729,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3D9386D-6B8B-45BB-B130-317C6F7A19D9}">
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="35.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="43.7109375" customWidth="1"/>
+    <col min="4" max="4" width="34.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -716,13 +746,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
         <v>49</v>
       </c>
       <c r="B3" s="18"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
         <v>51</v>
       </c>
@@ -730,15 +760,18 @@
         <v>20326225</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="18" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="B5" s="19">
+      <c r="B5" s="28">
         <v>20315513</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5" s="15" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
         <v>52</v>
       </c>
@@ -746,21 +779,24 @@
         <v>20302834</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
         <v>53</v>
       </c>
       <c r="B7" s="19">
         <v>20332883</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7" s="29" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B8" s="2"/>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
@@ -768,7 +804,7 @@
         <v>20324226</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>4</v>
       </c>
@@ -776,7 +812,7 @@
         <v>20324208</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
@@ -784,7 +820,7 @@
         <v>20334253</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>6</v>
       </c>
@@ -792,7 +828,7 @@
         <v>20328728</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>7</v>
       </c>
@@ -800,13 +836,13 @@
         <v>20328676</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B14" s="4"/>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>9</v>
       </c>
@@ -814,7 +850,7 @@
         <v>20335483</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>10</v>
       </c>
@@ -822,7 +858,7 @@
         <v>20303552</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>11</v>
       </c>
@@ -830,7 +866,7 @@
         <v>20305017</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>12</v>
       </c>
@@ -838,7 +874,7 @@
         <v>20299958</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>13</v>
       </c>
@@ -846,13 +882,13 @@
         <v>20296800</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>14</v>
       </c>
       <c r="B20" s="6"/>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>15</v>
       </c>
@@ -860,7 +896,7 @@
         <v>20297197</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>16</v>
       </c>
@@ -868,29 +904,35 @@
         <v>20305491</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B23" s="6">
         <v>20323047</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C23" s="29" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>18</v>
       </c>
       <c r="B24" s="6">
         <v>20332455</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C24" s="29" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>19</v>
       </c>
       <c r="B25" s="8"/>
     </row>
-    <row r="26" spans="1:2" s="25" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>50</v>
       </c>
@@ -898,7 +940,7 @@
         <v>20316171</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="24" t="s">
         <v>34</v>
       </c>
@@ -906,7 +948,7 @@
         <v>20326737</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>35</v>
       </c>
@@ -914,7 +956,7 @@
         <v>20334703</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
         <v>36</v>
       </c>
@@ -922,7 +964,7 @@
         <v>20304265</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>37</v>
       </c>
@@ -930,13 +972,13 @@
         <v>20299917</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B31" s="10"/>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
         <v>21</v>
       </c>
@@ -954,208 +996,226 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B34" s="10">
+        <v>20300963</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B34" s="10">
+      <c r="B35" s="10">
         <v>20301324</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="11" t="s">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B35" s="12"/>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="B36" s="12">
-        <v>20324308</v>
-      </c>
+      <c r="B36" s="12"/>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B37" s="12">
-        <v>20321372</v>
+        <v>20324308</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B38" s="12">
-        <v>20331182</v>
+        <v>20321372</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B39" s="12">
-        <v>20326560</v>
+        <v>20331182</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B40" s="12">
+        <v>20326560</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B40" s="12">
+      <c r="B41" s="12">
         <v>20343053</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="13" t="s">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="B41" s="14"/>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="B42" s="14">
-        <v>20331710</v>
-      </c>
+      <c r="B42" s="14"/>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B43" s="14">
-        <v>20338113</v>
+        <v>20331710</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B44" s="14">
+        <v>20338113</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B44" s="14">
+      <c r="B45" s="14">
         <v>20331094</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="21" t="s">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="B45" s="17"/>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="B46" s="17">
-        <v>20313810</v>
-      </c>
+      <c r="B46" s="17"/>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="17" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B47" s="17">
-        <v>20301942</v>
+        <v>20313810</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="B48" s="17">
+        <v>20301942</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="B48" s="17">
+      <c r="B49" s="17">
         <v>20305492</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" s="22" t="s">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="B50" s="27">
+        <v>20265699</v>
+      </c>
+      <c r="C50" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="B49" s="23"/>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="23" t="s">
+      <c r="B51" s="23"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="B50" s="23">
+      <c r="B52" s="23">
         <v>20325547</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51" s="23" t="s">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="B51" s="23">
+      <c r="B53" s="23">
         <v>20326271</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" s="23" t="s">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="B52" s="23">
+      <c r="B54" s="23">
         <v>20324344</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" s="23" t="s">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="B53" s="23">
+      <c r="B55" s="23">
         <v>20324307</v>
       </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" s="23" t="s">
+      <c r="C55" s="29" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="B54" s="23">
+      <c r="B56" s="23">
         <v>20346682</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55" s="16" t="s">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="B55" s="15"/>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="B56" s="15">
-        <v>20300963</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" s="15" t="s">
+      <c r="B57" s="15"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B57" s="15">
+      <c r="B59" s="15">
         <v>20177773</v>
       </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="B58" s="15">
-        <v>20265699</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" s="15" t="s">
+      <c r="C59" s="29" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B59" s="15">
+      <c r="B61" s="15">
         <v>20299200</v>
       </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" s="15" t="s">
+      <c r="C61" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="D61" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="B60" s="15">
+      <c r="B62" s="15">
         <v>20299004</v>
+      </c>
+      <c r="C62" s="29" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated GDV4000 list - added group work on repo so far
</commit_message>
<xml_diff>
--- a/T2/GDV4000/GDV4000_25_26_Groups.xlsx
+++ b/T2/GDV4000/GDV4000_25_26_Groups.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ian\TEACHING_25_26\2025_26\T2\GDV4000\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2476AA7C-ABEE-465A-97E3-97588E3E4E90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7504DE54-034B-4116-AA15-9745F51412C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="82440" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{587E5374-C9D8-4859-B380-F0EE43715D22}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="71">
   <si>
     <t>Team Member Name</t>
   </si>
@@ -98,9 +98,6 @@
     <t>The Blanks</t>
   </si>
   <si>
-    <t>TBC</t>
-  </si>
-  <si>
     <t>Rhys Sells</t>
   </si>
   <si>
@@ -225,13 +222,40 @@
   </si>
   <si>
     <t>Still awaiting to hear</t>
+  </si>
+  <si>
+    <t>No Content in repo apart from 10 page.</t>
+  </si>
+  <si>
+    <t>Only project, no GDD or Wiki.</t>
+  </si>
+  <si>
+    <t>NeonDash</t>
+  </si>
+  <si>
+    <t>GDD started and PRAC1</t>
+  </si>
+  <si>
+    <t>GDD in Wiki under development. No PRAC1 yet.</t>
+  </si>
+  <si>
+    <t>Olympia</t>
+  </si>
+  <si>
+    <t>Structure for GDD present. No evidence of PRAC1</t>
+  </si>
+  <si>
+    <t>Some evidence of PRAC1, but no WRIT1 or Wiki</t>
+  </si>
+  <si>
+    <t>No repo.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -254,8 +278,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -331,6 +362,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -356,7 +399,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -390,11 +433,15 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -735,10 +782,10 @@
     <col min="1" max="1" width="23.85546875" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="43.7109375" customWidth="1"/>
-    <col min="4" max="4" width="34.28515625" customWidth="1"/>
+    <col min="4" max="4" width="41.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -746,149 +793,163 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" s="18"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B4" s="19">
         <v>20326225</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="28">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="27">
         <v>20315513</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B6" s="19">
         <v>20302834</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B7" s="19">
         <v>20332883</v>
       </c>
-      <c r="C7" s="29" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C7" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B8" s="2"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B9" s="2">
         <v>20324226</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D9" s="33" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B10" s="2">
         <v>20324208</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D10" s="33"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B11" s="2">
         <v>20334253</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D11" s="33"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B12" s="2">
         <v>20328728</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D12" s="33"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="2">
         <v>20328676</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D13" s="33"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B14" s="4"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B15" s="4">
         <v>20335483</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D15" s="15" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="4">
         <v>20303552</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D16" s="15"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B17" s="4">
         <v>20305017</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D17" s="15"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B18" s="4">
         <v>20299958</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D18" s="15"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B19" s="4">
         <v>20296800</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D19" s="15"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>14</v>
       </c>
       <c r="B20" s="6"/>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>15</v>
       </c>
@@ -896,7 +957,7 @@
         <v>20297197</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>16</v>
       </c>
@@ -904,318 +965,352 @@
         <v>20305491</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B23" s="6">
         <v>20323047</v>
       </c>
-      <c r="C23" s="29" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C23" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>18</v>
       </c>
       <c r="B24" s="6">
         <v>20332455</v>
       </c>
-      <c r="C24" s="29" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C24" s="28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>19</v>
       </c>
       <c r="B25" s="8"/>
     </row>
-    <row r="26" spans="1:3" s="25" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B26" s="26">
         <v>20316171</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D26" s="31" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B27" s="24">
         <v>20326737</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D27" s="32"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B28" s="8">
         <v>20334703</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D28" s="32"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B29" s="8">
         <v>20304265</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D29" s="32"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B30" s="8">
         <v>20299917</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D30" s="32"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B31" s="10"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="10" t="s">
         <v>20</v>
-      </c>
-      <c r="B31" s="10"/>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="10" t="s">
-        <v>21</v>
       </c>
       <c r="B32" s="10">
         <v>20317343</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D32" s="33" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B33" s="10">
         <v>20304600</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D33" s="33"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B34" s="10">
         <v>20300963</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D34" s="33"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B35" s="10">
         <v>20301324</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D35" s="33"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B36" s="12"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="12" t="s">
         <v>24</v>
-      </c>
-      <c r="B36" s="12"/>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="12" t="s">
-        <v>25</v>
       </c>
       <c r="B37" s="12">
         <v>20324308</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D37" s="33" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B38" s="12">
         <v>20321372</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D38" s="33"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B39" s="12">
         <v>20331182</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D39" s="33"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B40" s="12">
         <v>20326560</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D40" s="33"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B41" s="12">
         <v>20343053</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D41" s="33"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B42" s="14"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="14" t="s">
         <v>30</v>
-      </c>
-      <c r="B42" s="14"/>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="14" t="s">
-        <v>31</v>
       </c>
       <c r="B43" s="14">
         <v>20331710</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B44" s="14">
         <v>20338113</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B45" s="14">
         <v>20331094</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B46" s="17"/>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D46" s="30" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B47" s="17">
         <v>20313810</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D47" s="29"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B48" s="17">
         <v>20301942</v>
       </c>
+      <c r="D48" s="29"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="17" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B49" s="17">
         <v>20305492</v>
       </c>
+      <c r="D49" s="29"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="27" t="s">
-        <v>41</v>
-      </c>
-      <c r="B50" s="27">
+      <c r="A50" t="s">
+        <v>40</v>
+      </c>
+      <c r="B50">
         <v>20265699</v>
       </c>
       <c r="C50" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="22" t="s">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="B51" s="23"/>
+      <c r="D51" s="30" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="23" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B52" s="23">
         <v>20325547</v>
       </c>
+      <c r="D52" s="15"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="23" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B53" s="23">
         <v>20326271</v>
       </c>
+      <c r="D53" s="15"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B54" s="23">
         <v>20324344</v>
       </c>
+      <c r="D54" s="15"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B55" s="23">
         <v>20324307</v>
       </c>
-      <c r="C55" s="29" t="s">
-        <v>60</v>
-      </c>
+      <c r="C55" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="D55" s="15"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B56" s="23">
         <v>20346682</v>
       </c>
+      <c r="D56" s="15"/>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B57" s="15"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B59" s="15">
         <v>20177773</v>
       </c>
-      <c r="C59" s="29" t="s">
-        <v>60</v>
+      <c r="C59" s="28" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B61" s="15">
         <v>20299200</v>
       </c>
-      <c r="C61" s="29" t="s">
+      <c r="C61" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="D61" t="s">
         <v>60</v>
-      </c>
-      <c r="D61" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B62" s="15">
         <v>20299004</v>
       </c>
-      <c r="C62" s="29" t="s">
-        <v>60</v>
+      <c r="C62" s="28" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Ethics for GDV4000 - One last look tomorrow, but should be ready
</commit_message>
<xml_diff>
--- a/T2/GDV4000/GDV4000_25_26_Groups.xlsx
+++ b/T2/GDV4000/GDV4000_25_26_Groups.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ian\TEACHING_25_26\2025_26\T2\GDV4000\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7504DE54-034B-4116-AA15-9745F51412C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCA70E6E-E1EF-4CB4-B764-3C30BA5CB2FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="82440" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{587E5374-C9D8-4859-B380-F0EE43715D22}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="72">
   <si>
     <t>Team Member Name</t>
   </si>
@@ -249,6 +249,9 @@
   </si>
   <si>
     <t>No repo.</t>
+  </si>
+  <si>
+    <t>Emailed 03/03/26 Lack of attendance</t>
   </si>
 </sst>
 </file>
@@ -399,7 +402,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -442,6 +445,7 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -825,6 +829,9 @@
       <c r="B6" s="19">
         <v>20302834</v>
       </c>
+      <c r="C6" s="34" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">

</xml_diff>

<commit_message>
Added folder structure for GDV4000 WRIT1 marking
</commit_message>
<xml_diff>
--- a/T2/GDV4000/GDV4000_25_26_Groups.xlsx
+++ b/T2/GDV4000/GDV4000_25_26_Groups.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ian\TEACHING_25_26\2025_26\T2\GDV4000\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCA70E6E-E1EF-4CB4-B764-3C30BA5CB2FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4950952-DC22-4E9E-BFB7-A7D9CD76507A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="82440" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{587E5374-C9D8-4859-B380-F0EE43715D22}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="74">
   <si>
     <t>Team Member Name</t>
   </si>
@@ -252,6 +252,12 @@
   </si>
   <si>
     <t>Emailed 03/03/26 Lack of attendance</t>
+  </si>
+  <si>
+    <t>WRIT1</t>
+  </si>
+  <si>
+    <t>PRAC1</t>
   </si>
 </sst>
 </file>
@@ -289,7 +295,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -376,7 +382,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -402,7 +414,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -445,7 +457,8 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -780,7 +793,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3D9386D-6B8B-45BB-B130-317C6F7A19D9}">
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" customWidth="1"/>
@@ -789,29 +802,39 @@
     <col min="4" max="4" width="41.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
         <v>48</v>
       </c>
       <c r="B3" s="18"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
         <v>50</v>
       </c>
       <c r="B4" s="19">
         <v>20326225</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>45</v>
       </c>
@@ -821,19 +844,23 @@
       <c r="C5" s="15" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
         <v>51</v>
       </c>
       <c r="B6" s="19">
         <v>20302834</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="14" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
         <v>52</v>
       </c>
@@ -843,67 +870,79 @@
       <c r="C7" s="28" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B8" s="2"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B9" s="2">
         <v>20324226</v>
       </c>
-      <c r="D9" s="33" t="s">
+      <c r="D9" s="14" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B10" s="2">
         <v>20324208</v>
       </c>
-      <c r="D10" s="33"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D10" s="14"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B11" s="2">
         <v>20334253</v>
       </c>
-      <c r="D11" s="33"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D11" s="14"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B12" s="2">
         <v>20328728</v>
       </c>
-      <c r="D12" s="33"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" s="14"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="2">
         <v>20328676</v>
       </c>
-      <c r="D13" s="33"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D13" s="14"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B14" s="4"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>9</v>
       </c>
@@ -913,8 +952,10 @@
       <c r="D15" s="15" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>10</v>
       </c>
@@ -922,8 +963,10 @@
         <v>20303552</v>
       </c>
       <c r="D16" s="15"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>11</v>
       </c>
@@ -931,8 +974,10 @@
         <v>20305017</v>
       </c>
       <c r="D17" s="15"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>12</v>
       </c>
@@ -940,8 +985,10 @@
         <v>20299958</v>
       </c>
       <c r="D18" s="15"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>13</v>
       </c>
@@ -949,30 +996,36 @@
         <v>20296800</v>
       </c>
       <c r="D19" s="15"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>14</v>
       </c>
       <c r="B20" s="6"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B21" s="6">
         <v>20297197</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>16</v>
       </c>
       <c r="B22" s="6">
         <v>20305491</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>17</v>
       </c>
@@ -982,8 +1035,10 @@
       <c r="C23" s="28" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>18</v>
       </c>
@@ -993,14 +1048,16 @@
       <c r="C24" s="28" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>19</v>
       </c>
       <c r="B25" s="8"/>
     </row>
-    <row r="26" spans="1:4" s="25" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" s="25" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>49</v>
       </c>
@@ -1010,8 +1067,10 @@
       <c r="D26" s="31" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="24" t="s">
         <v>33</v>
       </c>
@@ -1019,8 +1078,10 @@
         <v>20326737</v>
       </c>
       <c r="D27" s="32"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>34</v>
       </c>
@@ -1028,8 +1089,10 @@
         <v>20334703</v>
       </c>
       <c r="D28" s="32"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
         <v>35</v>
       </c>
@@ -1037,8 +1100,10 @@
         <v>20304265</v>
       </c>
       <c r="D29" s="32"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>36</v>
       </c>
@@ -1046,135 +1111,161 @@
         <v>20299917</v>
       </c>
       <c r="D30" s="32"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
         <v>67</v>
       </c>
       <c r="B31" s="10"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
         <v>20</v>
       </c>
       <c r="B32" s="10">
         <v>20317343</v>
       </c>
-      <c r="D32" s="33" t="s">
+      <c r="D32" s="14" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B33" s="10">
         <v>20304600</v>
       </c>
-      <c r="D33" s="33"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D33" s="14"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
         <v>37</v>
       </c>
       <c r="B34" s="10">
         <v>20300963</v>
       </c>
-      <c r="D34" s="33"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D34" s="14"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
         <v>22</v>
       </c>
       <c r="B35" s="10">
         <v>20301324</v>
       </c>
-      <c r="D35" s="33"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D35" s="14"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>23</v>
       </c>
       <c r="B36" s="12"/>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
         <v>24</v>
       </c>
       <c r="B37" s="12">
         <v>20324308</v>
       </c>
-      <c r="D37" s="33" t="s">
+      <c r="D37" s="14" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
         <v>25</v>
       </c>
       <c r="B38" s="12">
         <v>20321372</v>
       </c>
-      <c r="D38" s="33"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D38" s="14"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
         <v>26</v>
       </c>
       <c r="B39" s="12">
         <v>20331182</v>
       </c>
-      <c r="D39" s="33"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D39" s="14"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="12"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
         <v>27</v>
       </c>
       <c r="B40" s="12">
         <v>20326560</v>
       </c>
-      <c r="D40" s="33"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D40" s="14"/>
+      <c r="F40" s="12"/>
+      <c r="G40" s="12"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
         <v>28</v>
       </c>
       <c r="B41" s="12">
         <v>20343053</v>
       </c>
-      <c r="D41" s="33"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D41" s="14"/>
+      <c r="F41" s="12"/>
+      <c r="G41" s="12"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="13" t="s">
         <v>29</v>
       </c>
       <c r="B42" s="14"/>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
         <v>30</v>
       </c>
       <c r="B43" s="14">
         <v>20331710</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F43" s="14"/>
+      <c r="G43" s="14"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
         <v>31</v>
       </c>
       <c r="B44" s="14">
         <v>20338113</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F44" s="14"/>
+      <c r="G44" s="14"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
         <v>32</v>
       </c>
       <c r="B45" s="14">
         <v>20331094</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F45" s="14"/>
+      <c r="G45" s="14"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="21" t="s">
         <v>53</v>
       </c>
@@ -1183,7 +1274,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="17" t="s">
         <v>41</v>
       </c>
@@ -1191,8 +1282,10 @@
         <v>20313810</v>
       </c>
       <c r="D47" s="29"/>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F47" s="17"/>
+      <c r="G47" s="17"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="17" t="s">
         <v>47</v>
       </c>
@@ -1200,8 +1293,10 @@
         <v>20301942</v>
       </c>
       <c r="D48" s="29"/>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F48" s="17"/>
+      <c r="G48" s="17"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="17" t="s">
         <v>39</v>
       </c>
@@ -1209,116 +1304,138 @@
         <v>20305492</v>
       </c>
       <c r="D49" s="29"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>40</v>
-      </c>
-      <c r="B50">
-        <v>20265699</v>
-      </c>
-      <c r="C50" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="22" t="s">
+      <c r="F49" s="17"/>
+      <c r="G49" s="17"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="B51" s="23"/>
-      <c r="D51" s="30" t="s">
+      <c r="B50" s="23"/>
+      <c r="D50" s="30" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B51" s="23">
+        <v>20325547</v>
+      </c>
+      <c r="D51" s="15"/>
+      <c r="F51" s="23"/>
+      <c r="G51" s="23"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="23" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="B52" s="23">
-        <v>20325547</v>
+        <v>20326271</v>
       </c>
       <c r="D52" s="15"/>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F52" s="23"/>
+      <c r="G52" s="23"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="23" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B53" s="23">
-        <v>20326271</v>
+        <v>20324344</v>
       </c>
       <c r="D53" s="15"/>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F53" s="23"/>
+      <c r="G53" s="23"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="23" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B54" s="23">
-        <v>20324344</v>
+        <v>20324307</v>
+      </c>
+      <c r="C54" s="28" t="s">
+        <v>59</v>
       </c>
       <c r="D54" s="15"/>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F54" s="23"/>
+      <c r="G54" s="23"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B55" s="23">
-        <v>20324307</v>
-      </c>
-      <c r="C55" s="28" t="s">
+        <v>20346682</v>
+      </c>
+      <c r="D55" s="15"/>
+      <c r="F55" s="23"/>
+      <c r="G55" s="23"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="B56" s="15"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="B57" s="15">
+        <v>20177773</v>
+      </c>
+      <c r="C57" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="D55" s="15"/>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="B56" s="23">
-        <v>20346682</v>
-      </c>
-      <c r="D56" s="15"/>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B57" s="15"/>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F57" s="15"/>
+      <c r="G57" s="15"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B58" s="15">
+        <v>20299200</v>
+      </c>
+      <c r="C58" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="D58" t="s">
+        <v>60</v>
+      </c>
+      <c r="F58" s="15"/>
+      <c r="G58" s="15"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="15" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B59" s="15">
-        <v>20177773</v>
+        <v>20299004</v>
       </c>
       <c r="C59" s="28" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="B61" s="15">
-        <v>20299200</v>
-      </c>
-      <c r="C61" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="D61" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="B62" s="15">
-        <v>20299004</v>
-      </c>
-      <c r="C62" s="28" t="s">
-        <v>59</v>
-      </c>
+      <c r="F59" s="15"/>
+      <c r="G59" s="15"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="B60" s="35">
+        <v>20265699</v>
+      </c>
+      <c r="C60" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="D60" s="35"/>
+      <c r="E60" s="35"/>
+      <c r="F60" s="35"/>
+      <c r="G60" s="35"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated GDV4000 Marking Sheet. All marking done, IV3a shared with Glenn.
</commit_message>
<xml_diff>
--- a/T2/GDV4000/GDV4000_25_26_Groups.xlsx
+++ b/T2/GDV4000/GDV4000_25_26_Groups.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ian\TEACHING_25_26\2025_26\T2\GDV4000\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2025_26\T2\GDV4000\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4950952-DC22-4E9E-BFB7-A7D9CD76507A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE29CF0-1C27-4ECE-8A11-D069C3234F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="82440" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{587E5374-C9D8-4859-B380-F0EE43715D22}"/>
+    <workbookView xWindow="38410" yWindow="10" windowWidth="38380" windowHeight="20860" xr2:uid="{587E5374-C9D8-4859-B380-F0EE43715D22}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="84">
   <si>
     <t>Team Member Name</t>
   </si>
@@ -221,9 +221,6 @@
     <t>Responded - Has been ill but will be in.</t>
   </si>
   <si>
-    <t>Still awaiting to hear</t>
-  </si>
-  <si>
     <t>No Content in repo apart from 10 page.</t>
   </si>
   <si>
@@ -258,6 +255,39 @@
   </si>
   <si>
     <t>PRAC1</t>
+  </si>
+  <si>
+    <t>IV3a Changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Working indenpendently. </t>
+  </si>
+  <si>
+    <t>NS</t>
+  </si>
+  <si>
+    <t>Upper Second</t>
+  </si>
+  <si>
+    <t>First</t>
+  </si>
+  <si>
+    <t>Lower Second</t>
+  </si>
+  <si>
+    <t>Third</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>IV3a</t>
+  </si>
+  <si>
+    <t>NOTES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IV3a </t>
   </si>
 </sst>
 </file>
@@ -295,7 +325,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="23">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -389,6 +419,42 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -414,7 +480,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -436,9 +502,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -448,17 +511,89 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -793,93 +928,126 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3D9386D-6B8B-45BB-B130-317C6F7A19D9}">
-  <dimension ref="A1:G60"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I70"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" customWidth="1"/>
+    <col min="1" max="1" width="23.88671875" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="43.7109375" customWidth="1"/>
-    <col min="4" max="4" width="41.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.6640625" customWidth="1"/>
+    <col min="4" max="4" width="41.33203125" customWidth="1"/>
+    <col min="6" max="6" width="8.88671875" style="32"/>
+    <col min="7" max="7" width="12" style="32" customWidth="1"/>
+    <col min="8" max="8" width="8.88671875" style="32"/>
+    <col min="9" max="9" width="12.21875" style="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" t="s">
+      <c r="D1" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="G1" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="H1" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" s="32" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="20" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="19" t="s">
         <v>48</v>
       </c>
       <c r="B3" s="18"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="19">
+      <c r="B4" s="49">
         <v>20326225</v>
       </c>
-      <c r="F4" s="33"/>
-      <c r="G4" s="33"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="F4" s="50" t="s">
+        <v>75</v>
+      </c>
+      <c r="G4" s="46"/>
+      <c r="H4" s="33"/>
+      <c r="I4" s="46"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="27">
+      <c r="B5" s="56">
         <v>20315513</v>
       </c>
       <c r="C5" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="F5" s="34"/>
-      <c r="G5" s="34"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
+      <c r="E5" s="61" t="s">
+        <v>81</v>
+      </c>
+      <c r="F5" s="54">
+        <v>40</v>
+      </c>
+      <c r="G5" s="46"/>
+      <c r="H5" s="54"/>
+      <c r="I5" s="46"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="B6" s="19">
+      <c r="B6" s="49">
         <v>20302834</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="F6" s="50" t="s">
+        <v>75</v>
+      </c>
+      <c r="G6" s="46"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="46"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="B7" s="19">
+      <c r="B7" s="49">
         <v>20332883</v>
       </c>
-      <c r="C7" s="28" t="s">
+      <c r="C7" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="F7" s="33"/>
-      <c r="G7" s="33"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F7" s="50" t="s">
+        <v>75</v>
+      </c>
+      <c r="G7" s="46"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="46"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
@@ -887,12 +1055,16 @@
         <v>20324226</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+      <c r="F9" s="34">
+        <v>65</v>
+      </c>
+      <c r="G9" s="46"/>
+      <c r="H9" s="34"/>
+      <c r="I9" s="46"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>4</v>
       </c>
@@ -900,10 +1072,17 @@
         <v>20324208</v>
       </c>
       <c r="D10" s="14"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E10" s="63" t="s">
+        <v>81</v>
+      </c>
+      <c r="F10" s="34">
+        <v>67</v>
+      </c>
+      <c r="G10" s="46"/>
+      <c r="H10" s="34"/>
+      <c r="I10" s="46"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
@@ -911,10 +1090,14 @@
         <v>20334253</v>
       </c>
       <c r="D11" s="14"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F11" s="34">
+        <v>64</v>
+      </c>
+      <c r="G11" s="46"/>
+      <c r="H11" s="34"/>
+      <c r="I11" s="46"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>6</v>
       </c>
@@ -922,10 +1105,14 @@
         <v>20328728</v>
       </c>
       <c r="D12" s="14"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F12" s="34">
+        <v>66</v>
+      </c>
+      <c r="G12" s="46"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="46"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>7</v>
       </c>
@@ -933,16 +1120,20 @@
         <v>20328676</v>
       </c>
       <c r="D13" s="14"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F13" s="34">
+        <v>64</v>
+      </c>
+      <c r="G13" s="46"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="46"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B14" s="4"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>9</v>
       </c>
@@ -950,12 +1141,16 @@
         <v>20335483</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+      <c r="F15" s="35">
+        <v>69</v>
+      </c>
+      <c r="G15" s="46"/>
+      <c r="H15" s="35"/>
+      <c r="I15" s="46"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>10</v>
       </c>
@@ -963,10 +1158,14 @@
         <v>20303552</v>
       </c>
       <c r="D16" s="15"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F16" s="35">
+        <v>66</v>
+      </c>
+      <c r="G16" s="46"/>
+      <c r="H16" s="35"/>
+      <c r="I16" s="46"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>11</v>
       </c>
@@ -974,10 +1173,17 @@
         <v>20305017</v>
       </c>
       <c r="D17" s="15"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E17" s="63" t="s">
+        <v>81</v>
+      </c>
+      <c r="F17" s="35">
+        <v>69</v>
+      </c>
+      <c r="G17" s="46"/>
+      <c r="H17" s="35"/>
+      <c r="I17" s="46"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>12</v>
       </c>
@@ -985,10 +1191,14 @@
         <v>20299958</v>
       </c>
       <c r="D18" s="15"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F18" s="35">
+        <v>67</v>
+      </c>
+      <c r="G18" s="46"/>
+      <c r="H18" s="35"/>
+      <c r="I18" s="46"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>13</v>
       </c>
@@ -996,131 +1206,178 @@
         <v>20296800</v>
       </c>
       <c r="D19" s="15"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F19" s="35">
+        <v>68</v>
+      </c>
+      <c r="G19" s="46"/>
+      <c r="H19" s="35"/>
+      <c r="I19" s="46"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>14</v>
       </c>
       <c r="B20" s="6"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B21" s="6">
         <v>20297197</v>
       </c>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F21" s="36">
+        <v>41</v>
+      </c>
+      <c r="G21" s="46"/>
+      <c r="H21" s="36"/>
+      <c r="I21" s="46"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>16</v>
       </c>
       <c r="B22" s="6">
         <v>20305491</v>
       </c>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E22" s="61" t="s">
+        <v>81</v>
+      </c>
+      <c r="F22" s="36">
+        <v>41</v>
+      </c>
+      <c r="G22" s="46"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="46"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B23" s="6">
         <v>20323047</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F23" s="36">
+        <v>41</v>
+      </c>
+      <c r="G23" s="46"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="46"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>18</v>
       </c>
       <c r="B24" s="6">
         <v>20332455</v>
       </c>
-      <c r="C24" s="28" t="s">
+      <c r="C24" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E24" s="60"/>
+      <c r="F24" s="36">
+        <v>45</v>
+      </c>
+      <c r="G24" s="46"/>
+      <c r="H24" s="36"/>
+      <c r="I24" s="46"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
         <v>19</v>
       </c>
       <c r="B25" s="8"/>
     </row>
-    <row r="26" spans="1:7" s="25" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" s="24" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B26" s="26">
+      <c r="B26" s="25">
         <v>20316171</v>
       </c>
-      <c r="D26" s="31" t="s">
-        <v>65</v>
-      </c>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="24" t="s">
+      <c r="D26" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="F26" s="37">
+        <v>63</v>
+      </c>
+      <c r="G26" s="47"/>
+      <c r="H26" s="37"/>
+      <c r="I26" s="47"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="B27" s="24">
+      <c r="B27" s="23">
         <v>20326737</v>
       </c>
-      <c r="D27" s="32"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D27" s="30"/>
+      <c r="F27" s="38">
+        <v>66</v>
+      </c>
+      <c r="G27" s="46"/>
+      <c r="H27" s="38"/>
+      <c r="I27" s="46"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
         <v>34</v>
       </c>
       <c r="B28" s="8">
         <v>20334703</v>
       </c>
-      <c r="D28" s="32"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D28" s="30"/>
+      <c r="F28" s="38">
+        <v>66</v>
+      </c>
+      <c r="G28" s="46"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="46"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
         <v>35</v>
       </c>
       <c r="B29" s="8">
         <v>20304265</v>
       </c>
-      <c r="D29" s="32"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D29" s="30"/>
+      <c r="E29" s="63" t="s">
+        <v>81</v>
+      </c>
+      <c r="F29" s="38">
+        <v>63</v>
+      </c>
+      <c r="G29" s="46"/>
+      <c r="H29" s="38"/>
+      <c r="I29" s="46"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>36</v>
       </c>
       <c r="B30" s="8">
         <v>20299917</v>
       </c>
-      <c r="D30" s="32"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D30" s="30"/>
+      <c r="F30" s="38">
+        <v>66</v>
+      </c>
+      <c r="G30" s="46"/>
+      <c r="H30" s="38"/>
+      <c r="I30" s="46"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B31" s="10"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="10" t="s">
         <v>20</v>
       </c>
@@ -1128,12 +1385,16 @@
         <v>20317343</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="F32" s="39">
+        <v>70</v>
+      </c>
+      <c r="G32" s="46"/>
+      <c r="H32" s="39"/>
+      <c r="I32" s="46"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="10" t="s">
         <v>21</v>
       </c>
@@ -1141,21 +1402,32 @@
         <v>20304600</v>
       </c>
       <c r="D33" s="14"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="10" t="s">
+      <c r="E33" s="64" t="s">
+        <v>81</v>
+      </c>
+      <c r="F33" s="39">
+        <v>71</v>
+      </c>
+      <c r="G33" s="46"/>
+      <c r="H33" s="39"/>
+      <c r="I33" s="46"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A34" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="10">
+      <c r="B34" s="9">
         <v>20300963</v>
       </c>
       <c r="D34" s="14"/>
-      <c r="F34" s="10"/>
-      <c r="G34" s="10"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F34" s="51" t="s">
+        <v>75</v>
+      </c>
+      <c r="G34" s="46"/>
+      <c r="H34" s="39"/>
+      <c r="I34" s="46"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="10" t="s">
         <v>22</v>
       </c>
@@ -1163,16 +1435,20 @@
         <v>20301324</v>
       </c>
       <c r="D35" s="14"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F35" s="39">
+        <v>58</v>
+      </c>
+      <c r="G35" s="46"/>
+      <c r="H35" s="39"/>
+      <c r="I35" s="46"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
         <v>23</v>
       </c>
       <c r="B36" s="12"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="12" t="s">
         <v>24</v>
       </c>
@@ -1180,12 +1456,16 @@
         <v>20324308</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="F37" s="12"/>
-      <c r="G37" s="12"/>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+      <c r="F37" s="40">
+        <v>70</v>
+      </c>
+      <c r="G37" s="46"/>
+      <c r="H37" s="40"/>
+      <c r="I37" s="46"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="12" t="s">
         <v>25</v>
       </c>
@@ -1193,10 +1473,17 @@
         <v>20321372</v>
       </c>
       <c r="D38" s="14"/>
-      <c r="F38" s="12"/>
-      <c r="G38" s="12"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E38" s="64" t="s">
+        <v>81</v>
+      </c>
+      <c r="F38" s="40">
+        <v>73</v>
+      </c>
+      <c r="G38" s="46"/>
+      <c r="H38" s="40"/>
+      <c r="I38" s="46"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="12" t="s">
         <v>26</v>
       </c>
@@ -1204,10 +1491,17 @@
         <v>20331182</v>
       </c>
       <c r="D39" s="14"/>
-      <c r="F39" s="12"/>
-      <c r="G39" s="12"/>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E39" s="64" t="s">
+        <v>81</v>
+      </c>
+      <c r="F39" s="40">
+        <v>71</v>
+      </c>
+      <c r="G39" s="46"/>
+      <c r="H39" s="40"/>
+      <c r="I39" s="46"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="12" t="s">
         <v>27</v>
       </c>
@@ -1215,10 +1509,14 @@
         <v>20326560</v>
       </c>
       <c r="D40" s="14"/>
-      <c r="F40" s="12"/>
-      <c r="G40" s="12"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F40" s="40">
+        <v>67</v>
+      </c>
+      <c r="G40" s="46"/>
+      <c r="H40" s="40"/>
+      <c r="I40" s="46"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="12" t="s">
         <v>28</v>
       </c>
@@ -1226,216 +1524,353 @@
         <v>20343053</v>
       </c>
       <c r="D41" s="14"/>
-      <c r="F41" s="12"/>
-      <c r="G41" s="12"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F41" s="40">
+        <v>70</v>
+      </c>
+      <c r="G41" s="46"/>
+      <c r="H41" s="40"/>
+      <c r="I41" s="46"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="13" t="s">
         <v>29</v>
       </c>
       <c r="B42" s="14"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="14" t="s">
         <v>30</v>
       </c>
       <c r="B43" s="14">
         <v>20331710</v>
       </c>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F43" s="41">
+        <v>55</v>
+      </c>
+      <c r="G43" s="46"/>
+      <c r="H43" s="41"/>
+      <c r="I43" s="46"/>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="14" t="s">
         <v>31</v>
       </c>
       <c r="B44" s="14">
         <v>20338113</v>
       </c>
-      <c r="F44" s="14"/>
-      <c r="G44" s="14"/>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E44" s="62" t="s">
+        <v>81</v>
+      </c>
+      <c r="F44" s="41">
+        <v>56</v>
+      </c>
+      <c r="G44" s="46"/>
+      <c r="H44" s="41"/>
+      <c r="I44" s="46"/>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
         <v>32</v>
       </c>
       <c r="B45" s="14">
         <v>20331094</v>
       </c>
-      <c r="F45" s="14"/>
-      <c r="G45" s="14"/>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="21" t="s">
+      <c r="F45" s="41">
+        <v>57</v>
+      </c>
+      <c r="G45" s="46"/>
+      <c r="H45" s="41"/>
+      <c r="I45" s="46"/>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A46" s="20" t="s">
         <v>53</v>
       </c>
       <c r="B46" s="17"/>
-      <c r="D46" s="30" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D46" s="28" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="17" t="s">
         <v>41</v>
       </c>
       <c r="B47" s="17">
         <v>20313810</v>
       </c>
-      <c r="D47" s="29"/>
-      <c r="F47" s="17"/>
-      <c r="G47" s="17"/>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D47" s="27"/>
+      <c r="F47" s="42">
+        <v>52</v>
+      </c>
+      <c r="G47" s="46"/>
+      <c r="H47" s="42"/>
+      <c r="I47" s="46"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="17" t="s">
         <v>47</v>
       </c>
       <c r="B48" s="17">
         <v>20301942</v>
       </c>
-      <c r="D48" s="29"/>
-      <c r="F48" s="17"/>
-      <c r="G48" s="17"/>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D48" s="27"/>
+      <c r="E48" s="62" t="s">
+        <v>81</v>
+      </c>
+      <c r="F48" s="42">
+        <v>51</v>
+      </c>
+      <c r="G48" s="46"/>
+      <c r="H48" s="42"/>
+      <c r="I48" s="46"/>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="17" t="s">
         <v>39</v>
       </c>
       <c r="B49" s="17">
         <v>20305492</v>
       </c>
-      <c r="D49" s="29"/>
-      <c r="F49" s="17"/>
-      <c r="G49" s="17"/>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="22" t="s">
-        <v>64</v>
-      </c>
-      <c r="B50" s="23"/>
-      <c r="D50" s="30" t="s">
+      <c r="D49" s="27"/>
+      <c r="F49" s="42">
+        <v>53</v>
+      </c>
+      <c r="G49" s="46"/>
+      <c r="H49" s="42"/>
+      <c r="I49" s="46"/>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A50" s="21" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="23" t="s">
+      <c r="B50" s="22"/>
+      <c r="D50" s="28" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A51" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="B51" s="23">
+      <c r="B51" s="22">
         <v>20325547</v>
       </c>
       <c r="D51" s="15"/>
-      <c r="F51" s="23"/>
-      <c r="G51" s="23"/>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="23" t="s">
+      <c r="F51" s="43">
+        <v>45</v>
+      </c>
+      <c r="G51" s="46"/>
+      <c r="H51" s="43"/>
+      <c r="I51" s="46"/>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A52" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="B52" s="23">
+      <c r="B52" s="22">
         <v>20326271</v>
       </c>
       <c r="D52" s="15"/>
-      <c r="F52" s="23"/>
-      <c r="G52" s="23"/>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="23" t="s">
+      <c r="E52" s="61" t="s">
+        <v>81</v>
+      </c>
+      <c r="F52" s="43">
+        <v>47</v>
+      </c>
+      <c r="G52" s="46"/>
+      <c r="H52" s="43"/>
+      <c r="I52" s="46"/>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A53" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="B53" s="23">
+      <c r="B53" s="22">
         <v>20324344</v>
       </c>
       <c r="D53" s="15"/>
-      <c r="F53" s="23"/>
-      <c r="G53" s="23"/>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="23" t="s">
+      <c r="F53" s="43">
+        <v>46</v>
+      </c>
+      <c r="G53" s="46"/>
+      <c r="H53" s="43"/>
+      <c r="I53" s="46"/>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A54" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="B54" s="23">
+      <c r="B54" s="21">
         <v>20324307</v>
       </c>
-      <c r="C54" s="28" t="s">
+      <c r="C54" s="26" t="s">
         <v>59</v>
       </c>
       <c r="D54" s="15"/>
-      <c r="F54" s="23"/>
-      <c r="G54" s="23"/>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="23" t="s">
+      <c r="F54" s="53" t="s">
+        <v>75</v>
+      </c>
+      <c r="G54" s="46"/>
+      <c r="H54" s="43"/>
+      <c r="I54" s="46"/>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A55" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="B55" s="23">
+      <c r="B55" s="22">
         <v>20346682</v>
       </c>
       <c r="D55" s="15"/>
-      <c r="F55" s="23"/>
-      <c r="G55" s="23"/>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="16" t="s">
+      <c r="F55" s="43">
+        <v>47</v>
+      </c>
+      <c r="G55" s="46"/>
+      <c r="H55" s="43"/>
+      <c r="I55" s="46"/>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A57" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="B56" s="15"/>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="15" t="s">
+      <c r="B57" s="15"/>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A58" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="B57" s="15">
+      <c r="B58" s="52">
         <v>20177773</v>
       </c>
-      <c r="C57" s="28" t="s">
+      <c r="C58" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="F57" s="15"/>
-      <c r="G57" s="15"/>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="15" t="s">
+      <c r="F58" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="G58" s="46"/>
+      <c r="H58" s="44"/>
+      <c r="I58" s="46"/>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A59" s="52" t="s">
         <v>42</v>
       </c>
-      <c r="B58" s="15">
+      <c r="B59" s="52">
         <v>20299200</v>
       </c>
-      <c r="C58" s="28" t="s">
+      <c r="C59" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="D58" t="s">
+      <c r="D59" t="s">
         <v>60</v>
       </c>
-      <c r="F58" s="15"/>
-      <c r="G58" s="15"/>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" s="15" t="s">
+      <c r="F59" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="G59" s="46"/>
+      <c r="H59" s="44"/>
+      <c r="I59" s="46"/>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A60" s="52" t="s">
         <v>43</v>
       </c>
-      <c r="B59" s="15">
+      <c r="B60" s="52">
         <v>20299004</v>
       </c>
-      <c r="C59" s="28" t="s">
+      <c r="C60" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="F59" s="15"/>
-      <c r="G59" s="15"/>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="35" t="s">
+      <c r="F60" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="G60" s="46"/>
+      <c r="H60" s="44"/>
+      <c r="I60" s="46"/>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C61" s="48"/>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A62" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="B60" s="35">
+      <c r="B62" s="31">
         <v>20265699</v>
       </c>
-      <c r="C60" s="35" t="s">
-        <v>61</v>
-      </c>
-      <c r="D60" s="35"/>
-      <c r="E60" s="35"/>
-      <c r="F60" s="35"/>
-      <c r="G60" s="35"/>
+      <c r="C62" s="31" t="s">
+        <v>74</v>
+      </c>
+      <c r="D62" s="31"/>
+      <c r="E62" s="62" t="s">
+        <v>81</v>
+      </c>
+      <c r="F62" s="45">
+        <v>54</v>
+      </c>
+      <c r="G62" s="46"/>
+      <c r="H62" s="45"/>
+      <c r="I62" s="46"/>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="30" t="s">
+        <v>77</v>
+      </c>
+      <c r="B65" s="30"/>
+      <c r="C65">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="57" t="s">
+        <v>76</v>
+      </c>
+      <c r="B66" s="57"/>
+      <c r="C66">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="58" t="s">
+        <v>78</v>
+      </c>
+      <c r="B67" s="58"/>
+      <c r="C67">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B68" s="14"/>
+      <c r="C68">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="B69" s="15"/>
+      <c r="C69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70" s="59" t="s">
+        <v>75</v>
+      </c>
+      <c r="B70" s="59"/>
+      <c r="C70">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added IV for WRIT1 to excel sheet - All agreed
</commit_message>
<xml_diff>
--- a/T2/GDV4000/GDV4000_25_26_Groups.xlsx
+++ b/T2/GDV4000/GDV4000_25_26_Groups.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2025_26\T2\GDV4000\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE29CF0-1C27-4ECE-8A11-D069C3234F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EF0B973-E5C1-4708-9E92-D7E7A090804F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38410" yWindow="10" windowWidth="38380" windowHeight="20860" xr2:uid="{587E5374-C9D8-4859-B380-F0EE43715D22}"/>
+    <workbookView xWindow="22944" yWindow="0" windowWidth="23232" windowHeight="25296" xr2:uid="{587E5374-C9D8-4859-B380-F0EE43715D22}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="86">
   <si>
     <t>Team Member Name</t>
   </si>
@@ -288,6 +288,12 @@
   </si>
   <si>
     <t xml:space="preserve">IV3a </t>
+  </si>
+  <si>
+    <t>AGREED</t>
+  </si>
+  <si>
+    <t>NA</t>
   </si>
 </sst>
 </file>
@@ -983,7 +989,9 @@
       <c r="F4" s="50" t="s">
         <v>75</v>
       </c>
-      <c r="G4" s="46"/>
+      <c r="G4" s="46" t="s">
+        <v>85</v>
+      </c>
       <c r="H4" s="33"/>
       <c r="I4" s="46"/>
     </row>
@@ -1003,7 +1011,9 @@
       <c r="F5" s="54">
         <v>40</v>
       </c>
-      <c r="G5" s="46"/>
+      <c r="G5" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H5" s="54"/>
       <c r="I5" s="46"/>
     </row>
@@ -1020,7 +1030,9 @@
       <c r="F6" s="50" t="s">
         <v>75</v>
       </c>
-      <c r="G6" s="46"/>
+      <c r="G6" s="46" t="s">
+        <v>85</v>
+      </c>
       <c r="H6" s="33"/>
       <c r="I6" s="46"/>
     </row>
@@ -1037,7 +1049,9 @@
       <c r="F7" s="50" t="s">
         <v>75</v>
       </c>
-      <c r="G7" s="46"/>
+      <c r="G7" s="46" t="s">
+        <v>85</v>
+      </c>
       <c r="H7" s="33"/>
       <c r="I7" s="46"/>
     </row>
@@ -1060,7 +1074,9 @@
       <c r="F9" s="34">
         <v>65</v>
       </c>
-      <c r="G9" s="46"/>
+      <c r="G9" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H9" s="34"/>
       <c r="I9" s="46"/>
     </row>
@@ -1078,7 +1094,9 @@
       <c r="F10" s="34">
         <v>67</v>
       </c>
-      <c r="G10" s="46"/>
+      <c r="G10" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H10" s="34"/>
       <c r="I10" s="46"/>
     </row>
@@ -1093,7 +1111,9 @@
       <c r="F11" s="34">
         <v>64</v>
       </c>
-      <c r="G11" s="46"/>
+      <c r="G11" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H11" s="34"/>
       <c r="I11" s="46"/>
     </row>
@@ -1108,7 +1128,9 @@
       <c r="F12" s="34">
         <v>66</v>
       </c>
-      <c r="G12" s="46"/>
+      <c r="G12" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H12" s="34"/>
       <c r="I12" s="46"/>
     </row>
@@ -1123,7 +1145,9 @@
       <c r="F13" s="34">
         <v>64</v>
       </c>
-      <c r="G13" s="46"/>
+      <c r="G13" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H13" s="34"/>
       <c r="I13" s="46"/>
     </row>
@@ -1146,7 +1170,9 @@
       <c r="F15" s="35">
         <v>69</v>
       </c>
-      <c r="G15" s="46"/>
+      <c r="G15" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H15" s="35"/>
       <c r="I15" s="46"/>
     </row>
@@ -1161,7 +1187,9 @@
       <c r="F16" s="35">
         <v>66</v>
       </c>
-      <c r="G16" s="46"/>
+      <c r="G16" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H16" s="35"/>
       <c r="I16" s="46"/>
     </row>
@@ -1179,7 +1207,9 @@
       <c r="F17" s="35">
         <v>69</v>
       </c>
-      <c r="G17" s="46"/>
+      <c r="G17" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H17" s="35"/>
       <c r="I17" s="46"/>
     </row>
@@ -1194,7 +1224,9 @@
       <c r="F18" s="35">
         <v>67</v>
       </c>
-      <c r="G18" s="46"/>
+      <c r="G18" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H18" s="35"/>
       <c r="I18" s="46"/>
     </row>
@@ -1209,7 +1241,9 @@
       <c r="F19" s="35">
         <v>68</v>
       </c>
-      <c r="G19" s="46"/>
+      <c r="G19" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H19" s="35"/>
       <c r="I19" s="46"/>
     </row>
@@ -1229,7 +1263,9 @@
       <c r="F21" s="36">
         <v>41</v>
       </c>
-      <c r="G21" s="46"/>
+      <c r="G21" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H21" s="36"/>
       <c r="I21" s="46"/>
     </row>
@@ -1246,7 +1282,9 @@
       <c r="F22" s="36">
         <v>41</v>
       </c>
-      <c r="G22" s="46"/>
+      <c r="G22" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H22" s="36"/>
       <c r="I22" s="46"/>
     </row>
@@ -1263,7 +1301,9 @@
       <c r="F23" s="36">
         <v>41</v>
       </c>
-      <c r="G23" s="46"/>
+      <c r="G23" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H23" s="36"/>
       <c r="I23" s="46"/>
     </row>
@@ -1281,7 +1321,9 @@
       <c r="F24" s="36">
         <v>45</v>
       </c>
-      <c r="G24" s="46"/>
+      <c r="G24" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H24" s="36"/>
       <c r="I24" s="46"/>
     </row>
@@ -1304,7 +1346,9 @@
       <c r="F26" s="37">
         <v>63</v>
       </c>
-      <c r="G26" s="47"/>
+      <c r="G26" s="47" t="s">
+        <v>84</v>
+      </c>
       <c r="H26" s="37"/>
       <c r="I26" s="47"/>
     </row>
@@ -1319,7 +1363,9 @@
       <c r="F27" s="38">
         <v>66</v>
       </c>
-      <c r="G27" s="46"/>
+      <c r="G27" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H27" s="38"/>
       <c r="I27" s="46"/>
     </row>
@@ -1334,7 +1380,9 @@
       <c r="F28" s="38">
         <v>66</v>
       </c>
-      <c r="G28" s="46"/>
+      <c r="G28" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H28" s="38"/>
       <c r="I28" s="46"/>
     </row>
@@ -1352,7 +1400,9 @@
       <c r="F29" s="38">
         <v>63</v>
       </c>
-      <c r="G29" s="46"/>
+      <c r="G29" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H29" s="38"/>
       <c r="I29" s="46"/>
     </row>
@@ -1367,7 +1417,9 @@
       <c r="F30" s="38">
         <v>66</v>
       </c>
-      <c r="G30" s="46"/>
+      <c r="G30" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H30" s="38"/>
       <c r="I30" s="46"/>
     </row>
@@ -1390,7 +1442,9 @@
       <c r="F32" s="39">
         <v>70</v>
       </c>
-      <c r="G32" s="46"/>
+      <c r="G32" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H32" s="39"/>
       <c r="I32" s="46"/>
     </row>
@@ -1408,7 +1462,9 @@
       <c r="F33" s="39">
         <v>71</v>
       </c>
-      <c r="G33" s="46"/>
+      <c r="G33" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H33" s="39"/>
       <c r="I33" s="46"/>
     </row>
@@ -1423,7 +1479,9 @@
       <c r="F34" s="51" t="s">
         <v>75</v>
       </c>
-      <c r="G34" s="46"/>
+      <c r="G34" s="46" t="s">
+        <v>85</v>
+      </c>
       <c r="H34" s="39"/>
       <c r="I34" s="46"/>
     </row>
@@ -1438,7 +1496,9 @@
       <c r="F35" s="39">
         <v>58</v>
       </c>
-      <c r="G35" s="46"/>
+      <c r="G35" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H35" s="39"/>
       <c r="I35" s="46"/>
     </row>
@@ -1461,7 +1521,9 @@
       <c r="F37" s="40">
         <v>70</v>
       </c>
-      <c r="G37" s="46"/>
+      <c r="G37" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H37" s="40"/>
       <c r="I37" s="46"/>
     </row>
@@ -1479,7 +1541,9 @@
       <c r="F38" s="40">
         <v>73</v>
       </c>
-      <c r="G38" s="46"/>
+      <c r="G38" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H38" s="40"/>
       <c r="I38" s="46"/>
     </row>
@@ -1497,7 +1561,9 @@
       <c r="F39" s="40">
         <v>71</v>
       </c>
-      <c r="G39" s="46"/>
+      <c r="G39" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H39" s="40"/>
       <c r="I39" s="46"/>
     </row>
@@ -1512,7 +1578,9 @@
       <c r="F40" s="40">
         <v>67</v>
       </c>
-      <c r="G40" s="46"/>
+      <c r="G40" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H40" s="40"/>
       <c r="I40" s="46"/>
     </row>
@@ -1527,7 +1595,9 @@
       <c r="F41" s="40">
         <v>70</v>
       </c>
-      <c r="G41" s="46"/>
+      <c r="G41" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H41" s="40"/>
       <c r="I41" s="46"/>
     </row>
@@ -1547,7 +1617,9 @@
       <c r="F43" s="41">
         <v>55</v>
       </c>
-      <c r="G43" s="46"/>
+      <c r="G43" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H43" s="41"/>
       <c r="I43" s="46"/>
     </row>
@@ -1564,7 +1636,9 @@
       <c r="F44" s="41">
         <v>56</v>
       </c>
-      <c r="G44" s="46"/>
+      <c r="G44" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H44" s="41"/>
       <c r="I44" s="46"/>
     </row>
@@ -1578,7 +1652,9 @@
       <c r="F45" s="41">
         <v>57</v>
       </c>
-      <c r="G45" s="46"/>
+      <c r="G45" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H45" s="41"/>
       <c r="I45" s="46"/>
     </row>
@@ -1602,7 +1678,9 @@
       <c r="F47" s="42">
         <v>52</v>
       </c>
-      <c r="G47" s="46"/>
+      <c r="G47" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H47" s="42"/>
       <c r="I47" s="46"/>
     </row>
@@ -1620,7 +1698,9 @@
       <c r="F48" s="42">
         <v>51</v>
       </c>
-      <c r="G48" s="46"/>
+      <c r="G48" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H48" s="42"/>
       <c r="I48" s="46"/>
     </row>
@@ -1635,7 +1715,9 @@
       <c r="F49" s="42">
         <v>53</v>
       </c>
-      <c r="G49" s="46"/>
+      <c r="G49" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H49" s="42"/>
       <c r="I49" s="46"/>
     </row>
@@ -1659,7 +1741,9 @@
       <c r="F51" s="43">
         <v>45</v>
       </c>
-      <c r="G51" s="46"/>
+      <c r="G51" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H51" s="43"/>
       <c r="I51" s="46"/>
     </row>
@@ -1677,7 +1761,9 @@
       <c r="F52" s="43">
         <v>47</v>
       </c>
-      <c r="G52" s="46"/>
+      <c r="G52" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H52" s="43"/>
       <c r="I52" s="46"/>
     </row>
@@ -1692,7 +1778,9 @@
       <c r="F53" s="43">
         <v>46</v>
       </c>
-      <c r="G53" s="46"/>
+      <c r="G53" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H53" s="43"/>
       <c r="I53" s="46"/>
     </row>
@@ -1710,7 +1798,9 @@
       <c r="F54" s="53" t="s">
         <v>75</v>
       </c>
-      <c r="G54" s="46"/>
+      <c r="G54" s="46" t="s">
+        <v>85</v>
+      </c>
       <c r="H54" s="43"/>
       <c r="I54" s="46"/>
     </row>
@@ -1725,7 +1815,9 @@
       <c r="F55" s="43">
         <v>47</v>
       </c>
-      <c r="G55" s="46"/>
+      <c r="G55" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H55" s="43"/>
       <c r="I55" s="46"/>
     </row>
@@ -1748,7 +1840,9 @@
       <c r="F58" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="G58" s="46"/>
+      <c r="G58" s="46" t="s">
+        <v>85</v>
+      </c>
       <c r="H58" s="44"/>
       <c r="I58" s="46"/>
     </row>
@@ -1768,7 +1862,9 @@
       <c r="F59" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="G59" s="46"/>
+      <c r="G59" s="46" t="s">
+        <v>85</v>
+      </c>
       <c r="H59" s="44"/>
       <c r="I59" s="46"/>
     </row>
@@ -1785,7 +1881,9 @@
       <c r="F60" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="G60" s="46"/>
+      <c r="G60" s="46" t="s">
+        <v>85</v>
+      </c>
       <c r="H60" s="44"/>
       <c r="I60" s="46"/>
     </row>
@@ -1809,7 +1907,9 @@
       <c r="F62" s="45">
         <v>54</v>
       </c>
-      <c r="G62" s="46"/>
+      <c r="G62" s="46" t="s">
+        <v>84</v>
+      </c>
       <c r="H62" s="45"/>
       <c r="I62" s="46"/>
     </row>

</xml_diff>

<commit_message>
Added Reflective Reports for GDV4000
</commit_message>
<xml_diff>
--- a/T2/GDV4000/GDV4000_25_26_Groups.xlsx
+++ b/T2/GDV4000/GDV4000_25_26_Groups.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2025_26\T2\GDV4000\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Ian\TEACHING_25_26\2025_26\T2\GDV4000\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EF0B973-E5C1-4708-9E92-D7E7A090804F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22944" yWindow="0" windowWidth="23232" windowHeight="25296" xr2:uid="{587E5374-C9D8-4859-B380-F0EE43715D22}"/>
+    <workbookView xWindow="82440" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{587E5374-C9D8-4859-B380-F0EE43715D22}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -935,19 +935,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3D9386D-6B8B-45BB-B130-317C6F7A19D9}">
   <dimension ref="A1:I70"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="43.6640625" customWidth="1"/>
-    <col min="4" max="4" width="41.33203125" customWidth="1"/>
-    <col min="6" max="6" width="8.88671875" style="32"/>
+    <col min="3" max="3" width="43.7109375" customWidth="1"/>
+    <col min="4" max="4" width="41.28515625" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" style="32"/>
     <col min="7" max="7" width="12" style="32" customWidth="1"/>
-    <col min="8" max="8" width="8.88671875" style="32"/>
-    <col min="9" max="9" width="12.21875" style="32" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" style="32"/>
+    <col min="9" max="9" width="12.28515625" style="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -973,13 +973,13 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="19" t="s">
         <v>48</v>
       </c>
       <c r="B3" s="18"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>50</v>
       </c>
@@ -995,7 +995,7 @@
       <c r="H4" s="33"/>
       <c r="I4" s="46"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="55" t="s">
         <v>45</v>
       </c>
@@ -1017,7 +1017,7 @@
       <c r="H5" s="54"/>
       <c r="I5" s="46"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>51</v>
       </c>
@@ -1036,7 +1036,7 @@
       <c r="H6" s="33"/>
       <c r="I6" s="46"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>52</v>
       </c>
@@ -1055,13 +1055,13 @@
       <c r="H7" s="33"/>
       <c r="I7" s="46"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B8" s="2"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
@@ -1080,7 +1080,7 @@
       <c r="H9" s="34"/>
       <c r="I9" s="46"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>4</v>
       </c>
@@ -1100,7 +1100,7 @@
       <c r="H10" s="34"/>
       <c r="I10" s="46"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
@@ -1117,7 +1117,7 @@
       <c r="H11" s="34"/>
       <c r="I11" s="46"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>6</v>
       </c>
@@ -1134,7 +1134,7 @@
       <c r="H12" s="34"/>
       <c r="I12" s="46"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>7</v>
       </c>
@@ -1151,13 +1151,13 @@
       <c r="H13" s="34"/>
       <c r="I13" s="46"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B14" s="4"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>9</v>
       </c>
@@ -1176,7 +1176,7 @@
       <c r="H15" s="35"/>
       <c r="I15" s="46"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>10</v>
       </c>
@@ -1193,7 +1193,7 @@
       <c r="H16" s="35"/>
       <c r="I16" s="46"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>11</v>
       </c>
@@ -1213,7 +1213,7 @@
       <c r="H17" s="35"/>
       <c r="I17" s="46"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>12</v>
       </c>
@@ -1230,7 +1230,7 @@
       <c r="H18" s="35"/>
       <c r="I18" s="46"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>13</v>
       </c>
@@ -1247,13 +1247,13 @@
       <c r="H19" s="35"/>
       <c r="I19" s="46"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>14</v>
       </c>
       <c r="B20" s="6"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>15</v>
       </c>
@@ -1269,7 +1269,7 @@
       <c r="H21" s="36"/>
       <c r="I21" s="46"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>16</v>
       </c>
@@ -1288,7 +1288,7 @@
       <c r="H22" s="36"/>
       <c r="I22" s="46"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>17</v>
       </c>
@@ -1307,7 +1307,7 @@
       <c r="H23" s="36"/>
       <c r="I23" s="46"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>18</v>
       </c>
@@ -1327,13 +1327,13 @@
       <c r="H24" s="36"/>
       <c r="I24" s="46"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>19</v>
       </c>
       <c r="B25" s="8"/>
     </row>
-    <row r="26" spans="1:9" s="24" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" s="24" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>49</v>
       </c>
@@ -1352,7 +1352,7 @@
       <c r="H26" s="37"/>
       <c r="I26" s="47"/>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="23" t="s">
         <v>33</v>
       </c>
@@ -1369,7 +1369,7 @@
       <c r="H27" s="38"/>
       <c r="I27" s="46"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>34</v>
       </c>
@@ -1386,7 +1386,7 @@
       <c r="H28" s="38"/>
       <c r="I28" s="46"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
         <v>35</v>
       </c>
@@ -1406,7 +1406,7 @@
       <c r="H29" s="38"/>
       <c r="I29" s="46"/>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>36</v>
       </c>
@@ -1423,13 +1423,13 @@
       <c r="H30" s="38"/>
       <c r="I30" s="46"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
         <v>66</v>
       </c>
       <c r="B31" s="10"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
         <v>20</v>
       </c>
@@ -1448,7 +1448,7 @@
       <c r="H32" s="39"/>
       <c r="I32" s="46"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
         <v>21</v>
       </c>
@@ -1468,7 +1468,7 @@
       <c r="H33" s="39"/>
       <c r="I33" s="46"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
         <v>37</v>
       </c>
@@ -1485,7 +1485,7 @@
       <c r="H34" s="39"/>
       <c r="I34" s="46"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
         <v>22</v>
       </c>
@@ -1502,13 +1502,13 @@
       <c r="H35" s="39"/>
       <c r="I35" s="46"/>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>23</v>
       </c>
       <c r="B36" s="12"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
         <v>24</v>
       </c>
@@ -1527,7 +1527,7 @@
       <c r="H37" s="40"/>
       <c r="I37" s="46"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
         <v>25</v>
       </c>
@@ -1547,7 +1547,7 @@
       <c r="H38" s="40"/>
       <c r="I38" s="46"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
         <v>26</v>
       </c>
@@ -1567,7 +1567,7 @@
       <c r="H39" s="40"/>
       <c r="I39" s="46"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
         <v>27</v>
       </c>
@@ -1584,7 +1584,7 @@
       <c r="H40" s="40"/>
       <c r="I40" s="46"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
         <v>28</v>
       </c>
@@ -1601,13 +1601,13 @@
       <c r="H41" s="40"/>
       <c r="I41" s="46"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="13" t="s">
         <v>29</v>
       </c>
       <c r="B42" s="14"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
         <v>30</v>
       </c>
@@ -1623,7 +1623,7 @@
       <c r="H43" s="41"/>
       <c r="I43" s="46"/>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
         <v>31</v>
       </c>
@@ -1642,7 +1642,7 @@
       <c r="H44" s="41"/>
       <c r="I44" s="46"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
         <v>32</v>
       </c>
@@ -1658,7 +1658,7 @@
       <c r="H45" s="41"/>
       <c r="I45" s="46"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="20" t="s">
         <v>53</v>
       </c>
@@ -1667,7 +1667,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="17" t="s">
         <v>41</v>
       </c>
@@ -1684,7 +1684,7 @@
       <c r="H47" s="42"/>
       <c r="I47" s="46"/>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="17" t="s">
         <v>47</v>
       </c>
@@ -1704,7 +1704,7 @@
       <c r="H48" s="42"/>
       <c r="I48" s="46"/>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="17" t="s">
         <v>39</v>
       </c>
@@ -1721,7 +1721,7 @@
       <c r="H49" s="42"/>
       <c r="I49" s="46"/>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="21" t="s">
         <v>63</v>
       </c>
@@ -1730,7 +1730,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="22" t="s">
         <v>44</v>
       </c>
@@ -1747,7 +1747,7 @@
       <c r="H51" s="43"/>
       <c r="I51" s="46"/>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="22" t="s">
         <v>54</v>
       </c>
@@ -1767,7 +1767,7 @@
       <c r="H52" s="43"/>
       <c r="I52" s="46"/>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="22" t="s">
         <v>55</v>
       </c>
@@ -1784,7 +1784,7 @@
       <c r="H53" s="43"/>
       <c r="I53" s="46"/>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="21" t="s">
         <v>56</v>
       </c>
@@ -1804,7 +1804,7 @@
       <c r="H54" s="43"/>
       <c r="I54" s="46"/>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="22" t="s">
         <v>57</v>
       </c>
@@ -1821,13 +1821,13 @@
       <c r="H55" s="43"/>
       <c r="I55" s="46"/>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
         <v>46</v>
       </c>
       <c r="B57" s="15"/>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="52" t="s">
         <v>38</v>
       </c>
@@ -1846,7 +1846,7 @@
       <c r="H58" s="44"/>
       <c r="I58" s="46"/>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="52" t="s">
         <v>42</v>
       </c>
@@ -1868,7 +1868,7 @@
       <c r="H59" s="44"/>
       <c r="I59" s="46"/>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="52" t="s">
         <v>43</v>
       </c>
@@ -1887,10 +1887,10 @@
       <c r="H60" s="44"/>
       <c r="I60" s="46"/>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C61" s="48"/>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="31" t="s">
         <v>40</v>
       </c>
@@ -1913,12 +1913,12 @@
       <c r="H62" s="45"/>
       <c r="I62" s="46"/>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="30" t="s">
         <v>77</v>
       </c>
@@ -1927,7 +1927,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="57" t="s">
         <v>76</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="58" t="s">
         <v>78</v>
       </c>
@@ -1945,7 +1945,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
         <v>79</v>
       </c>
@@ -1954,7 +1954,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="15" t="s">
         <v>80</v>
       </c>
@@ -1963,7 +1963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="59" t="s">
         <v>75</v>
       </c>

</xml_diff>